<commit_message>
update Audio Naming Convention sheet
Bonus Symbol sounds
</commit_message>
<xml_diff>
--- a/AudioNamingConvention.xlsx
+++ b/AudioNamingConvention.xlsx
@@ -5,10 +5,10 @@
   <workbookPr date1904="1" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gtechcorp-my.sharepoint.com/personal/kristin_miltner_igt_com/Documents/Playa/Docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miltnek/igtinteractive/slot-template-audio-howler/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="114_{36351BCD-0DEF-0A47-AB8B-B9DFCCFCB1AD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{10CC98B0-9954-7B41-9DF8-C697C820BBC0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F02127-D59C-3640-92CB-A78ECBE2A3FE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="24440" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -166,15 +166,6 @@
     <t>Play this when the symbols first tumble after the play field has been cleared. Do not use this for successive individual tumbles after a win (see onTumbleXLand) This is a sound mockup of all the impact sfx of the symbols tumbling. Start this sound when the first symbol in column 1 hits the bottom left corner of the playfield, not after the bounce. Alternatively these sounds can be grouped by the columns the symbols are falling in. For example onTumble2Start would play when the bottom most symbol in the second column hits the bottom of the playfield. Use this sound only for the bottom most symbols, the other symbol sounds will be mocked by the sfx.</t>
   </si>
   <si>
-    <t>onBonusSymbolS01Win
-onBonusSymbolS02Win
-onBonus2SymbolS03Win
-onBonusSymbolS04Win
-onBonusSymbolS05Win
-onBonusSymbolS06Win
-onBonusSymbolS07Win​           onBonusSymbolW01Win</t>
-  </si>
-  <si>
     <t xml:space="preserve">Same direction as onSymbolXXXWin but in the bonus. For multiple bonuses append the bonus number after the word Bonus, e.g. </t>
   </si>
   <si>
@@ -798,6 +789,15 @@
 onSymbolWinS05
 onSymbolWinS06
 onSymbolWinS07</t>
+  </si>
+  <si>
+    <t>onBonusSymbolWinS01
+onBonusSymbolWinS02
+onBonus2SymbolWinS03
+onBonusSymbolWinS04
+onBonusSymbolWinS05
+onBonusSymbolWinS06
+onBonusSymbolWinS07​           onBonusSymbolWinW01</t>
   </si>
 </sst>
 </file>
@@ -1103,13 +1103,13 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="4" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -2314,19 +2314,19 @@
   <sheetData>
     <row r="1" spans="1:252" ht="14" x14ac:dyDescent="0.15">
       <c r="A1" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="16" t="s">
-        <v>93</v>
-      </c>
       <c r="C1" s="37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:252" ht="14" x14ac:dyDescent="0.15">
       <c r="A2" s="27" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
@@ -2334,70 +2334,70 @@
     </row>
     <row r="3" spans="1:252" ht="14" x14ac:dyDescent="0.15">
       <c r="A3" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C3" s="39" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D3" s="14"/>
     </row>
     <row r="4" spans="1:252" ht="14" x14ac:dyDescent="0.15">
       <c r="A4" s="17" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C4" s="39" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D4" s="14"/>
     </row>
     <row r="5" spans="1:252" ht="28" x14ac:dyDescent="0.15">
       <c r="A5" s="17" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:252" ht="17" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="17" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C6" s="39" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D6" s="14"/>
     </row>
     <row r="7" spans="1:252" ht="16" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="17" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C7" s="39" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:252" ht="70" x14ac:dyDescent="0.15">
       <c r="A8" s="17" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>2</v>
@@ -2406,10 +2406,10 @@
     </row>
     <row r="9" spans="1:252" ht="70" x14ac:dyDescent="0.15">
       <c r="A9" s="17" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C9" s="40" t="s">
         <v>37</v>
@@ -2418,79 +2418,79 @@
     </row>
     <row r="10" spans="1:252" ht="42" x14ac:dyDescent="0.15">
       <c r="A10" s="17" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D10" s="14"/>
     </row>
     <row r="11" spans="1:252" ht="34" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="B11" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="C11" s="40" t="s">
         <v>240</v>
-      </c>
-      <c r="C11" s="40" t="s">
-        <v>241</v>
       </c>
       <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:252" ht="98" x14ac:dyDescent="0.15">
       <c r="A12" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C12" s="39" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D12" s="14"/>
     </row>
     <row r="13" spans="1:252" ht="70" x14ac:dyDescent="0.15">
       <c r="A13" s="17" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C13" s="39" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D13" s="14"/>
     </row>
     <row r="14" spans="1:252" ht="70" x14ac:dyDescent="0.15">
       <c r="A14" s="17" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B14" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>236</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="D14" s="14"/>
     </row>
     <row r="15" spans="1:252" ht="42" x14ac:dyDescent="0.15">
       <c r="A15" s="17" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D15" s="14"/>
     </row>
     <row r="16" spans="1:252" s="36" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="33" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B16" s="58" t="s">
         <v>32</v>
@@ -2750,7 +2750,7 @@
     </row>
     <row r="17" spans="1:252" s="36" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="33" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B17" s="58" t="s">
         <v>34</v>
@@ -3264,13 +3264,13 @@
     </row>
     <row r="19" spans="1:252" s="36" customFormat="1" ht="102" x14ac:dyDescent="0.2">
       <c r="A19" s="33" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D19" s="34"/>
       <c r="E19" s="35"/>
@@ -3524,13 +3524,13 @@
     </row>
     <row r="20" spans="1:252" s="36" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B20" s="32" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C20" s="41" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D20" s="34"/>
       <c r="E20" s="35"/>
@@ -3784,7 +3784,7 @@
     </row>
     <row r="21" spans="1:252" ht="14" x14ac:dyDescent="0.15">
       <c r="A21" s="27" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B21" s="27"/>
       <c r="C21" s="44"/>
@@ -3792,10 +3792,10 @@
     </row>
     <row r="22" spans="1:252" ht="42" x14ac:dyDescent="0.15">
       <c r="A22" s="17" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C22" s="39" t="s">
         <v>38</v>
@@ -3804,29 +3804,29 @@
     </row>
     <row r="23" spans="1:252" ht="28" x14ac:dyDescent="0.15">
       <c r="A23" s="17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C23" s="38"/>
       <c r="D23" s="14"/>
     </row>
     <row r="24" spans="1:252" ht="28" x14ac:dyDescent="0.15">
       <c r="A24" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C24" s="39" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D24" s="14"/>
     </row>
     <row r="25" spans="1:252" x14ac:dyDescent="0.15">
       <c r="A25" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="44"/>
@@ -3834,13 +3834,13 @@
     </row>
     <row r="26" spans="1:252" s="31" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" s="28" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B26" s="32" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C26" s="41" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D26" s="29"/>
       <c r="E26" s="30"/>
@@ -4094,10 +4094,10 @@
     </row>
     <row r="27" spans="1:252" s="31" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="28" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C27" s="41" t="s">
         <v>39</v>
@@ -4354,22 +4354,22 @@
     </row>
     <row r="28" spans="1:252" ht="28" x14ac:dyDescent="0.15">
       <c r="A28" s="25" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B28" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="44" t="s">
         <v>51</v>
-      </c>
-      <c r="C28" s="44" t="s">
-        <v>52</v>
       </c>
       <c r="D28" s="14"/>
     </row>
     <row r="29" spans="1:252" ht="14" x14ac:dyDescent="0.15">
       <c r="A29" s="17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B29" s="60" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C29" s="61" t="s">
         <v>36</v>
@@ -4378,32 +4378,32 @@
     </row>
     <row r="30" spans="1:252" ht="14" x14ac:dyDescent="0.15">
       <c r="A30" s="17" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C30" s="39"/>
       <c r="D30" s="14"/>
     </row>
     <row r="31" spans="1:252" ht="56" x14ac:dyDescent="0.15">
       <c r="A31" s="17" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C31" s="39" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D31" s="14"/>
     </row>
     <row r="32" spans="1:252" ht="28" x14ac:dyDescent="0.15">
       <c r="A32" s="17" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C32" s="39" t="s">
         <v>40</v>
@@ -4412,31 +4412,31 @@
     </row>
     <row r="33" spans="1:252" ht="98" x14ac:dyDescent="0.15">
       <c r="A33" s="17" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B33" s="18" t="s">
+        <v>246</v>
+      </c>
+      <c r="C33" s="39" t="s">
         <v>45</v>
-      </c>
-      <c r="C33" s="39" t="s">
-        <v>46</v>
       </c>
       <c r="D33" s="14"/>
     </row>
     <row r="34" spans="1:252" ht="14" x14ac:dyDescent="0.15">
       <c r="A34" s="17" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C34" s="39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D34" s="14"/>
     </row>
     <row r="35" spans="1:252" x14ac:dyDescent="0.15">
       <c r="A35" s="23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B35" s="24"/>
       <c r="C35" s="42"/>
@@ -4444,15 +4444,15 @@
     </row>
     <row r="36" spans="1:252" ht="14" x14ac:dyDescent="0.15">
       <c r="A36" s="17" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B36" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="C36" s="63" t="s">
         <v>70</v>
       </c>
-      <c r="C36" s="64" t="s">
-        <v>71</v>
-      </c>
-      <c r="D36" s="63"/>
+      <c r="D36" s="65"/>
       <c r="E36" s="62"/>
       <c r="F36" s="62"/>
       <c r="G36" s="62"/>
@@ -4707,8 +4707,8 @@
       <c r="B37" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="C37" s="65"/>
-      <c r="D37" s="63"/>
+      <c r="C37" s="64"/>
+      <c r="D37" s="65"/>
       <c r="E37" s="62"/>
       <c r="F37" s="62"/>
       <c r="G37" s="62"/>
@@ -4963,8 +4963,8 @@
       <c r="B38" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C38" s="65"/>
-      <c r="D38" s="63"/>
+      <c r="C38" s="64"/>
+      <c r="D38" s="65"/>
       <c r="E38" s="62"/>
       <c r="F38" s="62"/>
       <c r="G38" s="62"/>
@@ -5219,8 +5219,8 @@
       <c r="B39" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C39" s="65"/>
-      <c r="D39" s="63"/>
+      <c r="C39" s="64"/>
+      <c r="D39" s="65"/>
       <c r="E39" s="62"/>
       <c r="F39" s="62"/>
       <c r="G39" s="62"/>
@@ -5472,10 +5472,10 @@
     </row>
     <row r="40" spans="1:252" ht="98" x14ac:dyDescent="0.15">
       <c r="A40" s="17" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C40" s="39" t="s">
         <v>44</v>
@@ -5484,25 +5484,25 @@
     </row>
     <row r="41" spans="1:252" ht="28" x14ac:dyDescent="0.15">
       <c r="A41" s="17" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C41" s="38" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D41" s="14"/>
     </row>
     <row r="42" spans="1:252" ht="28" x14ac:dyDescent="0.15">
       <c r="A42" s="17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B42" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="C42" s="38" t="s">
         <v>75</v>
-      </c>
-      <c r="C42" s="38" t="s">
-        <v>76</v>
       </c>
       <c r="D42" s="14"/>
     </row>
@@ -5516,7 +5516,7 @@
     </row>
     <row r="44" spans="1:252" ht="14" x14ac:dyDescent="0.15">
       <c r="A44" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B44" s="22" t="s">
         <v>10</v>
@@ -5524,7 +5524,7 @@
       <c r="C44" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="D44" s="63"/>
+      <c r="D44" s="65"/>
       <c r="E44" s="62"/>
       <c r="F44" s="62"/>
       <c r="G44" s="62"/>
@@ -5776,7 +5776,7 @@
     </row>
     <row r="45" spans="1:252" ht="16" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="17" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B45" s="22" t="s">
         <v>11</v>
@@ -5784,7 +5784,7 @@
       <c r="C45" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="D45" s="63"/>
+      <c r="D45" s="65"/>
       <c r="E45" s="62"/>
       <c r="F45" s="62"/>
       <c r="G45" s="62"/>
@@ -6036,7 +6036,7 @@
     </row>
     <row r="46" spans="1:252" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="17" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B46" s="22" t="s">
         <v>12</v>
@@ -6044,7 +6044,7 @@
       <c r="C46" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="D46" s="63"/>
+      <c r="D46" s="65"/>
       <c r="E46" s="62"/>
       <c r="F46" s="62"/>
       <c r="G46" s="62"/>
@@ -6296,7 +6296,7 @@
     </row>
     <row r="47" spans="1:252" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="17" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B47" s="22" t="s">
         <v>13</v>
@@ -6304,7 +6304,7 @@
       <c r="C47" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="D47" s="63"/>
+      <c r="D47" s="65"/>
       <c r="E47" s="62"/>
       <c r="F47" s="62"/>
       <c r="G47" s="62"/>
@@ -6556,7 +6556,7 @@
     </row>
     <row r="48" spans="1:252" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="17" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B48" s="22" t="s">
         <v>14</v>
@@ -6816,7 +6816,7 @@
     </row>
     <row r="49" spans="1:252" ht="16" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="17" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B49" s="22" t="s">
         <v>22</v>
@@ -7076,7 +7076,7 @@
     </row>
     <row r="50" spans="1:252" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="17" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B50" s="22" t="s">
         <v>15</v>
@@ -7336,7 +7336,7 @@
     </row>
     <row r="51" spans="1:252" ht="16" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="17" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B51" s="22" t="s">
         <v>16</v>
@@ -7596,7 +7596,7 @@
     </row>
     <row r="52" spans="1:252" ht="16" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="17" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B52" s="22" t="s">
         <v>17</v>
@@ -7856,7 +7856,7 @@
     </row>
     <row r="53" spans="1:252" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="17" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B53" s="22" t="s">
         <v>18</v>
@@ -8116,7 +8116,7 @@
     </row>
     <row r="54" spans="1:252" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="17" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B54" s="22" t="s">
         <v>19</v>
@@ -8376,7 +8376,7 @@
     </row>
     <row r="55" spans="1:252" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="17" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B55" s="22" t="s">
         <v>20</v>
@@ -8636,7 +8636,7 @@
     </row>
     <row r="56" spans="1:252" ht="16" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="17" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B56" s="22" t="s">
         <v>21</v>
@@ -8896,7 +8896,7 @@
     </row>
     <row r="57" spans="1:252" ht="35" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>0</v>
@@ -9156,7 +9156,7 @@
     </row>
     <row r="58" spans="1:252" ht="16" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="23" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B58" s="24"/>
       <c r="C58" s="42"/>
@@ -9164,13 +9164,13 @@
     </row>
     <row r="59" spans="1:252" ht="35" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="17" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D59" s="51"/>
       <c r="E59" s="50"/>
@@ -9424,13 +9424,13 @@
     </row>
     <row r="60" spans="1:252" ht="35" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="17" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D60" s="51"/>
       <c r="E60" s="50"/>
@@ -9684,13 +9684,13 @@
     </row>
     <row r="61" spans="1:252" ht="35" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" s="17" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B61" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C61" s="3" t="s">
         <v>179</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>180</v>
       </c>
       <c r="D61" s="51"/>
       <c r="E61" s="50"/>
@@ -9944,13 +9944,13 @@
     </row>
     <row r="62" spans="1:252" ht="35" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" s="17" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D62" s="51"/>
       <c r="E62" s="50"/>
@@ -10204,13 +10204,13 @@
     </row>
     <row r="63" spans="1:252" ht="35" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A63" s="17" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D63" s="51"/>
       <c r="E63" s="50"/>
@@ -10464,7 +10464,7 @@
     </row>
     <row r="64" spans="1:252" ht="14" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A64" s="55" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B64" s="56"/>
       <c r="C64" s="56"/>
@@ -10733,489 +10733,6 @@
     </row>
   </sheetData>
   <mergeCells count="499">
-    <mergeCell ref="IN36:IN39"/>
-    <mergeCell ref="IO36:IO39"/>
-    <mergeCell ref="IP36:IP39"/>
-    <mergeCell ref="IQ36:IQ39"/>
-    <mergeCell ref="IR36:IR39"/>
-    <mergeCell ref="IH36:IH39"/>
-    <mergeCell ref="II36:II39"/>
-    <mergeCell ref="IJ36:IJ39"/>
-    <mergeCell ref="IK36:IK39"/>
-    <mergeCell ref="IL36:IL39"/>
-    <mergeCell ref="IM36:IM39"/>
-    <mergeCell ref="IB36:IB39"/>
-    <mergeCell ref="IC36:IC39"/>
-    <mergeCell ref="ID36:ID39"/>
-    <mergeCell ref="IE36:IE39"/>
-    <mergeCell ref="IF36:IF39"/>
-    <mergeCell ref="IG36:IG39"/>
-    <mergeCell ref="HV36:HV39"/>
-    <mergeCell ref="HW36:HW39"/>
-    <mergeCell ref="HX36:HX39"/>
-    <mergeCell ref="HY36:HY39"/>
-    <mergeCell ref="HZ36:HZ39"/>
-    <mergeCell ref="IA36:IA39"/>
-    <mergeCell ref="HP36:HP39"/>
-    <mergeCell ref="HQ36:HQ39"/>
-    <mergeCell ref="HR36:HR39"/>
-    <mergeCell ref="HS36:HS39"/>
-    <mergeCell ref="HT36:HT39"/>
-    <mergeCell ref="HU36:HU39"/>
-    <mergeCell ref="HJ36:HJ39"/>
-    <mergeCell ref="HK36:HK39"/>
-    <mergeCell ref="HL36:HL39"/>
-    <mergeCell ref="HM36:HM39"/>
-    <mergeCell ref="HN36:HN39"/>
-    <mergeCell ref="HO36:HO39"/>
-    <mergeCell ref="HD36:HD39"/>
-    <mergeCell ref="HE36:HE39"/>
-    <mergeCell ref="HF36:HF39"/>
-    <mergeCell ref="HG36:HG39"/>
-    <mergeCell ref="HH36:HH39"/>
-    <mergeCell ref="HI36:HI39"/>
-    <mergeCell ref="GX36:GX39"/>
-    <mergeCell ref="GY36:GY39"/>
-    <mergeCell ref="GZ36:GZ39"/>
-    <mergeCell ref="HA36:HA39"/>
-    <mergeCell ref="HB36:HB39"/>
-    <mergeCell ref="HC36:HC39"/>
-    <mergeCell ref="GR36:GR39"/>
-    <mergeCell ref="GS36:GS39"/>
-    <mergeCell ref="GT36:GT39"/>
-    <mergeCell ref="GU36:GU39"/>
-    <mergeCell ref="GV36:GV39"/>
-    <mergeCell ref="GW36:GW39"/>
-    <mergeCell ref="GL36:GL39"/>
-    <mergeCell ref="GM36:GM39"/>
-    <mergeCell ref="GN36:GN39"/>
-    <mergeCell ref="GO36:GO39"/>
-    <mergeCell ref="GP36:GP39"/>
-    <mergeCell ref="GQ36:GQ39"/>
-    <mergeCell ref="GF36:GF39"/>
-    <mergeCell ref="GG36:GG39"/>
-    <mergeCell ref="GH36:GH39"/>
-    <mergeCell ref="GI36:GI39"/>
-    <mergeCell ref="GJ36:GJ39"/>
-    <mergeCell ref="GK36:GK39"/>
-    <mergeCell ref="FZ36:FZ39"/>
-    <mergeCell ref="GA36:GA39"/>
-    <mergeCell ref="GB36:GB39"/>
-    <mergeCell ref="GC36:GC39"/>
-    <mergeCell ref="GD36:GD39"/>
-    <mergeCell ref="GE36:GE39"/>
-    <mergeCell ref="FT36:FT39"/>
-    <mergeCell ref="FU36:FU39"/>
-    <mergeCell ref="FV36:FV39"/>
-    <mergeCell ref="FW36:FW39"/>
-    <mergeCell ref="FX36:FX39"/>
-    <mergeCell ref="FY36:FY39"/>
-    <mergeCell ref="FN36:FN39"/>
-    <mergeCell ref="FO36:FO39"/>
-    <mergeCell ref="FP36:FP39"/>
-    <mergeCell ref="FQ36:FQ39"/>
-    <mergeCell ref="FR36:FR39"/>
-    <mergeCell ref="FS36:FS39"/>
-    <mergeCell ref="FH36:FH39"/>
-    <mergeCell ref="FI36:FI39"/>
-    <mergeCell ref="FJ36:FJ39"/>
-    <mergeCell ref="FK36:FK39"/>
-    <mergeCell ref="FL36:FL39"/>
-    <mergeCell ref="FM36:FM39"/>
-    <mergeCell ref="FB36:FB39"/>
-    <mergeCell ref="FC36:FC39"/>
-    <mergeCell ref="FD36:FD39"/>
-    <mergeCell ref="FE36:FE39"/>
-    <mergeCell ref="FF36:FF39"/>
-    <mergeCell ref="FG36:FG39"/>
-    <mergeCell ref="EV36:EV39"/>
-    <mergeCell ref="EW36:EW39"/>
-    <mergeCell ref="EX36:EX39"/>
-    <mergeCell ref="EY36:EY39"/>
-    <mergeCell ref="EZ36:EZ39"/>
-    <mergeCell ref="FA36:FA39"/>
-    <mergeCell ref="EP36:EP39"/>
-    <mergeCell ref="EQ36:EQ39"/>
-    <mergeCell ref="ER36:ER39"/>
-    <mergeCell ref="ES36:ES39"/>
-    <mergeCell ref="ET36:ET39"/>
-    <mergeCell ref="EU36:EU39"/>
-    <mergeCell ref="EJ36:EJ39"/>
-    <mergeCell ref="EK36:EK39"/>
-    <mergeCell ref="EL36:EL39"/>
-    <mergeCell ref="EM36:EM39"/>
-    <mergeCell ref="EN36:EN39"/>
-    <mergeCell ref="EO36:EO39"/>
-    <mergeCell ref="ED36:ED39"/>
-    <mergeCell ref="EE36:EE39"/>
-    <mergeCell ref="EF36:EF39"/>
-    <mergeCell ref="EG36:EG39"/>
-    <mergeCell ref="EH36:EH39"/>
-    <mergeCell ref="EI36:EI39"/>
-    <mergeCell ref="DX36:DX39"/>
-    <mergeCell ref="DY36:DY39"/>
-    <mergeCell ref="DZ36:DZ39"/>
-    <mergeCell ref="EA36:EA39"/>
-    <mergeCell ref="EB36:EB39"/>
-    <mergeCell ref="EC36:EC39"/>
-    <mergeCell ref="DR36:DR39"/>
-    <mergeCell ref="DS36:DS39"/>
-    <mergeCell ref="DT36:DT39"/>
-    <mergeCell ref="DU36:DU39"/>
-    <mergeCell ref="DV36:DV39"/>
-    <mergeCell ref="DW36:DW39"/>
-    <mergeCell ref="DL36:DL39"/>
-    <mergeCell ref="DM36:DM39"/>
-    <mergeCell ref="DN36:DN39"/>
-    <mergeCell ref="DO36:DO39"/>
-    <mergeCell ref="DP36:DP39"/>
-    <mergeCell ref="DQ36:DQ39"/>
-    <mergeCell ref="DF36:DF39"/>
-    <mergeCell ref="DG36:DG39"/>
-    <mergeCell ref="DH36:DH39"/>
-    <mergeCell ref="DI36:DI39"/>
-    <mergeCell ref="DJ36:DJ39"/>
-    <mergeCell ref="DK36:DK39"/>
-    <mergeCell ref="CZ36:CZ39"/>
-    <mergeCell ref="DA36:DA39"/>
-    <mergeCell ref="DB36:DB39"/>
-    <mergeCell ref="DC36:DC39"/>
-    <mergeCell ref="DD36:DD39"/>
-    <mergeCell ref="DE36:DE39"/>
-    <mergeCell ref="CT36:CT39"/>
-    <mergeCell ref="CU36:CU39"/>
-    <mergeCell ref="CV36:CV39"/>
-    <mergeCell ref="CW36:CW39"/>
-    <mergeCell ref="CX36:CX39"/>
-    <mergeCell ref="CY36:CY39"/>
-    <mergeCell ref="CN36:CN39"/>
-    <mergeCell ref="CO36:CO39"/>
-    <mergeCell ref="CP36:CP39"/>
-    <mergeCell ref="CQ36:CQ39"/>
-    <mergeCell ref="CR36:CR39"/>
-    <mergeCell ref="CS36:CS39"/>
-    <mergeCell ref="CH36:CH39"/>
-    <mergeCell ref="CI36:CI39"/>
-    <mergeCell ref="CJ36:CJ39"/>
-    <mergeCell ref="CK36:CK39"/>
-    <mergeCell ref="CL36:CL39"/>
-    <mergeCell ref="CM36:CM39"/>
-    <mergeCell ref="CB36:CB39"/>
-    <mergeCell ref="CC36:CC39"/>
-    <mergeCell ref="CD36:CD39"/>
-    <mergeCell ref="CE36:CE39"/>
-    <mergeCell ref="CF36:CF39"/>
-    <mergeCell ref="CG36:CG39"/>
-    <mergeCell ref="BV36:BV39"/>
-    <mergeCell ref="BW36:BW39"/>
-    <mergeCell ref="BX36:BX39"/>
-    <mergeCell ref="BY36:BY39"/>
-    <mergeCell ref="BZ36:BZ39"/>
-    <mergeCell ref="CA36:CA39"/>
-    <mergeCell ref="BP36:BP39"/>
-    <mergeCell ref="BQ36:BQ39"/>
-    <mergeCell ref="BR36:BR39"/>
-    <mergeCell ref="BS36:BS39"/>
-    <mergeCell ref="BT36:BT39"/>
-    <mergeCell ref="BU36:BU39"/>
-    <mergeCell ref="BJ36:BJ39"/>
-    <mergeCell ref="BK36:BK39"/>
-    <mergeCell ref="BL36:BL39"/>
-    <mergeCell ref="BM36:BM39"/>
-    <mergeCell ref="BN36:BN39"/>
-    <mergeCell ref="BO36:BO39"/>
-    <mergeCell ref="BD36:BD39"/>
-    <mergeCell ref="BE36:BE39"/>
-    <mergeCell ref="BF36:BF39"/>
-    <mergeCell ref="BG36:BG39"/>
-    <mergeCell ref="BH36:BH39"/>
-    <mergeCell ref="BI36:BI39"/>
-    <mergeCell ref="AX36:AX39"/>
-    <mergeCell ref="AY36:AY39"/>
-    <mergeCell ref="AZ36:AZ39"/>
-    <mergeCell ref="BA36:BA39"/>
-    <mergeCell ref="BB36:BB39"/>
-    <mergeCell ref="BC36:BC39"/>
-    <mergeCell ref="AR36:AR39"/>
-    <mergeCell ref="AS36:AS39"/>
-    <mergeCell ref="AT36:AT39"/>
-    <mergeCell ref="AU36:AU39"/>
-    <mergeCell ref="AV36:AV39"/>
-    <mergeCell ref="AW36:AW39"/>
-    <mergeCell ref="AL36:AL39"/>
-    <mergeCell ref="AM36:AM39"/>
-    <mergeCell ref="AN36:AN39"/>
-    <mergeCell ref="AO36:AO39"/>
-    <mergeCell ref="AP36:AP39"/>
-    <mergeCell ref="AQ36:AQ39"/>
-    <mergeCell ref="AF36:AF39"/>
-    <mergeCell ref="AG36:AG39"/>
-    <mergeCell ref="AH36:AH39"/>
-    <mergeCell ref="AI36:AI39"/>
-    <mergeCell ref="AJ36:AJ39"/>
-    <mergeCell ref="AK36:AK39"/>
-    <mergeCell ref="Z36:Z39"/>
-    <mergeCell ref="AA36:AA39"/>
-    <mergeCell ref="AB36:AB39"/>
-    <mergeCell ref="AC36:AC39"/>
-    <mergeCell ref="AD36:AD39"/>
-    <mergeCell ref="AE36:AE39"/>
-    <mergeCell ref="V36:V39"/>
-    <mergeCell ref="W36:W39"/>
-    <mergeCell ref="X36:X39"/>
-    <mergeCell ref="Y36:Y39"/>
-    <mergeCell ref="N36:N39"/>
-    <mergeCell ref="O36:O39"/>
-    <mergeCell ref="P36:P39"/>
-    <mergeCell ref="Q36:Q39"/>
-    <mergeCell ref="R36:R39"/>
-    <mergeCell ref="S36:S39"/>
-    <mergeCell ref="L36:L39"/>
-    <mergeCell ref="M36:M39"/>
-    <mergeCell ref="C36:C39"/>
-    <mergeCell ref="D36:D39"/>
-    <mergeCell ref="E36:E39"/>
-    <mergeCell ref="F36:F39"/>
-    <mergeCell ref="G36:G39"/>
-    <mergeCell ref="T36:T39"/>
-    <mergeCell ref="U36:U39"/>
-    <mergeCell ref="D44:D47"/>
-    <mergeCell ref="E44:E47"/>
-    <mergeCell ref="F44:F47"/>
-    <mergeCell ref="G44:G47"/>
-    <mergeCell ref="H44:H47"/>
-    <mergeCell ref="I44:I47"/>
-    <mergeCell ref="J44:J47"/>
-    <mergeCell ref="K44:K47"/>
-    <mergeCell ref="H36:H39"/>
-    <mergeCell ref="I36:I39"/>
-    <mergeCell ref="J36:J39"/>
-    <mergeCell ref="K36:K39"/>
-    <mergeCell ref="L44:L47"/>
-    <mergeCell ref="M44:M47"/>
-    <mergeCell ref="N44:N47"/>
-    <mergeCell ref="O44:O47"/>
-    <mergeCell ref="P44:P47"/>
-    <mergeCell ref="Q44:Q47"/>
-    <mergeCell ref="R44:R47"/>
-    <mergeCell ref="S44:S47"/>
-    <mergeCell ref="T44:T47"/>
-    <mergeCell ref="U44:U47"/>
-    <mergeCell ref="V44:V47"/>
-    <mergeCell ref="W44:W47"/>
-    <mergeCell ref="X44:X47"/>
-    <mergeCell ref="Y44:Y47"/>
-    <mergeCell ref="Z44:Z47"/>
-    <mergeCell ref="AA44:AA47"/>
-    <mergeCell ref="AB44:AB47"/>
-    <mergeCell ref="AC44:AC47"/>
-    <mergeCell ref="AD44:AD47"/>
-    <mergeCell ref="AE44:AE47"/>
-    <mergeCell ref="AF44:AF47"/>
-    <mergeCell ref="AG44:AG47"/>
-    <mergeCell ref="AH44:AH47"/>
-    <mergeCell ref="AI44:AI47"/>
-    <mergeCell ref="AJ44:AJ47"/>
-    <mergeCell ref="AK44:AK47"/>
-    <mergeCell ref="AL44:AL47"/>
-    <mergeCell ref="AM44:AM47"/>
-    <mergeCell ref="AN44:AN47"/>
-    <mergeCell ref="AO44:AO47"/>
-    <mergeCell ref="AP44:AP47"/>
-    <mergeCell ref="AQ44:AQ47"/>
-    <mergeCell ref="AR44:AR47"/>
-    <mergeCell ref="AS44:AS47"/>
-    <mergeCell ref="AT44:AT47"/>
-    <mergeCell ref="AU44:AU47"/>
-    <mergeCell ref="AV44:AV47"/>
-    <mergeCell ref="AW44:AW47"/>
-    <mergeCell ref="AX44:AX47"/>
-    <mergeCell ref="AY44:AY47"/>
-    <mergeCell ref="AZ44:AZ47"/>
-    <mergeCell ref="BA44:BA47"/>
-    <mergeCell ref="BB44:BB47"/>
-    <mergeCell ref="BC44:BC47"/>
-    <mergeCell ref="BD44:BD47"/>
-    <mergeCell ref="BE44:BE47"/>
-    <mergeCell ref="BF44:BF47"/>
-    <mergeCell ref="BG44:BG47"/>
-    <mergeCell ref="BH44:BH47"/>
-    <mergeCell ref="BI44:BI47"/>
-    <mergeCell ref="BJ44:BJ47"/>
-    <mergeCell ref="BK44:BK47"/>
-    <mergeCell ref="BL44:BL47"/>
-    <mergeCell ref="BM44:BM47"/>
-    <mergeCell ref="BN44:BN47"/>
-    <mergeCell ref="BO44:BO47"/>
-    <mergeCell ref="BP44:BP47"/>
-    <mergeCell ref="BQ44:BQ47"/>
-    <mergeCell ref="BR44:BR47"/>
-    <mergeCell ref="BS44:BS47"/>
-    <mergeCell ref="BT44:BT47"/>
-    <mergeCell ref="BU44:BU47"/>
-    <mergeCell ref="BV44:BV47"/>
-    <mergeCell ref="BW44:BW47"/>
-    <mergeCell ref="BX44:BX47"/>
-    <mergeCell ref="BY44:BY47"/>
-    <mergeCell ref="BZ44:BZ47"/>
-    <mergeCell ref="CA44:CA47"/>
-    <mergeCell ref="CB44:CB47"/>
-    <mergeCell ref="CC44:CC47"/>
-    <mergeCell ref="CD44:CD47"/>
-    <mergeCell ref="CE44:CE47"/>
-    <mergeCell ref="CF44:CF47"/>
-    <mergeCell ref="CG44:CG47"/>
-    <mergeCell ref="CH44:CH47"/>
-    <mergeCell ref="CI44:CI47"/>
-    <mergeCell ref="CJ44:CJ47"/>
-    <mergeCell ref="CK44:CK47"/>
-    <mergeCell ref="CL44:CL47"/>
-    <mergeCell ref="CM44:CM47"/>
-    <mergeCell ref="CN44:CN47"/>
-    <mergeCell ref="CO44:CO47"/>
-    <mergeCell ref="CP44:CP47"/>
-    <mergeCell ref="CQ44:CQ47"/>
-    <mergeCell ref="CR44:CR47"/>
-    <mergeCell ref="CS44:CS47"/>
-    <mergeCell ref="CT44:CT47"/>
-    <mergeCell ref="CU44:CU47"/>
-    <mergeCell ref="CV44:CV47"/>
-    <mergeCell ref="CW44:CW47"/>
-    <mergeCell ref="CX44:CX47"/>
-    <mergeCell ref="CY44:CY47"/>
-    <mergeCell ref="CZ44:CZ47"/>
-    <mergeCell ref="DA44:DA47"/>
-    <mergeCell ref="DB44:DB47"/>
-    <mergeCell ref="DC44:DC47"/>
-    <mergeCell ref="DD44:DD47"/>
-    <mergeCell ref="DE44:DE47"/>
-    <mergeCell ref="DF44:DF47"/>
-    <mergeCell ref="DG44:DG47"/>
-    <mergeCell ref="DH44:DH47"/>
-    <mergeCell ref="DI44:DI47"/>
-    <mergeCell ref="DJ44:DJ47"/>
-    <mergeCell ref="DK44:DK47"/>
-    <mergeCell ref="DL44:DL47"/>
-    <mergeCell ref="DM44:DM47"/>
-    <mergeCell ref="DN44:DN47"/>
-    <mergeCell ref="DO44:DO47"/>
-    <mergeCell ref="DP44:DP47"/>
-    <mergeCell ref="DQ44:DQ47"/>
-    <mergeCell ref="DR44:DR47"/>
-    <mergeCell ref="DS44:DS47"/>
-    <mergeCell ref="DT44:DT47"/>
-    <mergeCell ref="DU44:DU47"/>
-    <mergeCell ref="DV44:DV47"/>
-    <mergeCell ref="DW44:DW47"/>
-    <mergeCell ref="DX44:DX47"/>
-    <mergeCell ref="DY44:DY47"/>
-    <mergeCell ref="DZ44:DZ47"/>
-    <mergeCell ref="EA44:EA47"/>
-    <mergeCell ref="EB44:EB47"/>
-    <mergeCell ref="EC44:EC47"/>
-    <mergeCell ref="ED44:ED47"/>
-    <mergeCell ref="EE44:EE47"/>
-    <mergeCell ref="EF44:EF47"/>
-    <mergeCell ref="EG44:EG47"/>
-    <mergeCell ref="EH44:EH47"/>
-    <mergeCell ref="EI44:EI47"/>
-    <mergeCell ref="EJ44:EJ47"/>
-    <mergeCell ref="EK44:EK47"/>
-    <mergeCell ref="EL44:EL47"/>
-    <mergeCell ref="EM44:EM47"/>
-    <mergeCell ref="EN44:EN47"/>
-    <mergeCell ref="EO44:EO47"/>
-    <mergeCell ref="EP44:EP47"/>
-    <mergeCell ref="EQ44:EQ47"/>
-    <mergeCell ref="ER44:ER47"/>
-    <mergeCell ref="ES44:ES47"/>
-    <mergeCell ref="ET44:ET47"/>
-    <mergeCell ref="EU44:EU47"/>
-    <mergeCell ref="EV44:EV47"/>
-    <mergeCell ref="EW44:EW47"/>
-    <mergeCell ref="EX44:EX47"/>
-    <mergeCell ref="EY44:EY47"/>
-    <mergeCell ref="EZ44:EZ47"/>
-    <mergeCell ref="FA44:FA47"/>
-    <mergeCell ref="FB44:FB47"/>
-    <mergeCell ref="FC44:FC47"/>
-    <mergeCell ref="FD44:FD47"/>
-    <mergeCell ref="FE44:FE47"/>
-    <mergeCell ref="FF44:FF47"/>
-    <mergeCell ref="FG44:FG47"/>
-    <mergeCell ref="FH44:FH47"/>
-    <mergeCell ref="FI44:FI47"/>
-    <mergeCell ref="FJ44:FJ47"/>
-    <mergeCell ref="FK44:FK47"/>
-    <mergeCell ref="FL44:FL47"/>
-    <mergeCell ref="FM44:FM47"/>
-    <mergeCell ref="FN44:FN47"/>
-    <mergeCell ref="FO44:FO47"/>
-    <mergeCell ref="FP44:FP47"/>
-    <mergeCell ref="FQ44:FQ47"/>
-    <mergeCell ref="FR44:FR47"/>
-    <mergeCell ref="FS44:FS47"/>
-    <mergeCell ref="FT44:FT47"/>
-    <mergeCell ref="FU44:FU47"/>
-    <mergeCell ref="FV44:FV47"/>
-    <mergeCell ref="FW44:FW47"/>
-    <mergeCell ref="FX44:FX47"/>
-    <mergeCell ref="FY44:FY47"/>
-    <mergeCell ref="FZ44:FZ47"/>
-    <mergeCell ref="GA44:GA47"/>
-    <mergeCell ref="GB44:GB47"/>
-    <mergeCell ref="GC44:GC47"/>
-    <mergeCell ref="GD44:GD47"/>
-    <mergeCell ref="GE44:GE47"/>
-    <mergeCell ref="GF44:GF47"/>
-    <mergeCell ref="GG44:GG47"/>
-    <mergeCell ref="GH44:GH47"/>
-    <mergeCell ref="GI44:GI47"/>
-    <mergeCell ref="GJ44:GJ47"/>
-    <mergeCell ref="GK44:GK47"/>
-    <mergeCell ref="GL44:GL47"/>
-    <mergeCell ref="GM44:GM47"/>
-    <mergeCell ref="GN44:GN47"/>
-    <mergeCell ref="GO44:GO47"/>
-    <mergeCell ref="GP44:GP47"/>
-    <mergeCell ref="GQ44:GQ47"/>
-    <mergeCell ref="GR44:GR47"/>
-    <mergeCell ref="GS44:GS47"/>
-    <mergeCell ref="GT44:GT47"/>
-    <mergeCell ref="GU44:GU47"/>
-    <mergeCell ref="GV44:GV47"/>
-    <mergeCell ref="GW44:GW47"/>
-    <mergeCell ref="GX44:GX47"/>
-    <mergeCell ref="GY44:GY47"/>
-    <mergeCell ref="GZ44:GZ47"/>
-    <mergeCell ref="HA44:HA47"/>
-    <mergeCell ref="HB44:HB47"/>
-    <mergeCell ref="HC44:HC47"/>
-    <mergeCell ref="HD44:HD47"/>
-    <mergeCell ref="HE44:HE47"/>
-    <mergeCell ref="HF44:HF47"/>
-    <mergeCell ref="HG44:HG47"/>
-    <mergeCell ref="HH44:HH47"/>
-    <mergeCell ref="HI44:HI47"/>
-    <mergeCell ref="HJ44:HJ47"/>
-    <mergeCell ref="HK44:HK47"/>
-    <mergeCell ref="HL44:HL47"/>
-    <mergeCell ref="HM44:HM47"/>
-    <mergeCell ref="HN44:HN47"/>
-    <mergeCell ref="HO44:HO47"/>
-    <mergeCell ref="HP44:HP47"/>
-    <mergeCell ref="HQ44:HQ47"/>
-    <mergeCell ref="HR44:HR47"/>
-    <mergeCell ref="HS44:HS47"/>
-    <mergeCell ref="HT44:HT47"/>
-    <mergeCell ref="HU44:HU47"/>
-    <mergeCell ref="HV44:HV47"/>
-    <mergeCell ref="HW44:HW47"/>
-    <mergeCell ref="HX44:HX47"/>
-    <mergeCell ref="HY44:HY47"/>
-    <mergeCell ref="HZ44:HZ47"/>
-    <mergeCell ref="IA44:IA47"/>
-    <mergeCell ref="IB44:IB47"/>
     <mergeCell ref="IL44:IL47"/>
     <mergeCell ref="IM44:IM47"/>
     <mergeCell ref="IN44:IN47"/>
@@ -11232,6 +10749,489 @@
     <mergeCell ref="II44:II47"/>
     <mergeCell ref="IJ44:IJ47"/>
     <mergeCell ref="IK44:IK47"/>
+    <mergeCell ref="HT44:HT47"/>
+    <mergeCell ref="HU44:HU47"/>
+    <mergeCell ref="HV44:HV47"/>
+    <mergeCell ref="HW44:HW47"/>
+    <mergeCell ref="HX44:HX47"/>
+    <mergeCell ref="HY44:HY47"/>
+    <mergeCell ref="HZ44:HZ47"/>
+    <mergeCell ref="IA44:IA47"/>
+    <mergeCell ref="IB44:IB47"/>
+    <mergeCell ref="HK44:HK47"/>
+    <mergeCell ref="HL44:HL47"/>
+    <mergeCell ref="HM44:HM47"/>
+    <mergeCell ref="HN44:HN47"/>
+    <mergeCell ref="HO44:HO47"/>
+    <mergeCell ref="HP44:HP47"/>
+    <mergeCell ref="HQ44:HQ47"/>
+    <mergeCell ref="HR44:HR47"/>
+    <mergeCell ref="HS44:HS47"/>
+    <mergeCell ref="HB44:HB47"/>
+    <mergeCell ref="HC44:HC47"/>
+    <mergeCell ref="HD44:HD47"/>
+    <mergeCell ref="HE44:HE47"/>
+    <mergeCell ref="HF44:HF47"/>
+    <mergeCell ref="HG44:HG47"/>
+    <mergeCell ref="HH44:HH47"/>
+    <mergeCell ref="HI44:HI47"/>
+    <mergeCell ref="HJ44:HJ47"/>
+    <mergeCell ref="GS44:GS47"/>
+    <mergeCell ref="GT44:GT47"/>
+    <mergeCell ref="GU44:GU47"/>
+    <mergeCell ref="GV44:GV47"/>
+    <mergeCell ref="GW44:GW47"/>
+    <mergeCell ref="GX44:GX47"/>
+    <mergeCell ref="GY44:GY47"/>
+    <mergeCell ref="GZ44:GZ47"/>
+    <mergeCell ref="HA44:HA47"/>
+    <mergeCell ref="GJ44:GJ47"/>
+    <mergeCell ref="GK44:GK47"/>
+    <mergeCell ref="GL44:GL47"/>
+    <mergeCell ref="GM44:GM47"/>
+    <mergeCell ref="GN44:GN47"/>
+    <mergeCell ref="GO44:GO47"/>
+    <mergeCell ref="GP44:GP47"/>
+    <mergeCell ref="GQ44:GQ47"/>
+    <mergeCell ref="GR44:GR47"/>
+    <mergeCell ref="GA44:GA47"/>
+    <mergeCell ref="GB44:GB47"/>
+    <mergeCell ref="GC44:GC47"/>
+    <mergeCell ref="GD44:GD47"/>
+    <mergeCell ref="GE44:GE47"/>
+    <mergeCell ref="GF44:GF47"/>
+    <mergeCell ref="GG44:GG47"/>
+    <mergeCell ref="GH44:GH47"/>
+    <mergeCell ref="GI44:GI47"/>
+    <mergeCell ref="FR44:FR47"/>
+    <mergeCell ref="FS44:FS47"/>
+    <mergeCell ref="FT44:FT47"/>
+    <mergeCell ref="FU44:FU47"/>
+    <mergeCell ref="FV44:FV47"/>
+    <mergeCell ref="FW44:FW47"/>
+    <mergeCell ref="FX44:FX47"/>
+    <mergeCell ref="FY44:FY47"/>
+    <mergeCell ref="FZ44:FZ47"/>
+    <mergeCell ref="FI44:FI47"/>
+    <mergeCell ref="FJ44:FJ47"/>
+    <mergeCell ref="FK44:FK47"/>
+    <mergeCell ref="FL44:FL47"/>
+    <mergeCell ref="FM44:FM47"/>
+    <mergeCell ref="FN44:FN47"/>
+    <mergeCell ref="FO44:FO47"/>
+    <mergeCell ref="FP44:FP47"/>
+    <mergeCell ref="FQ44:FQ47"/>
+    <mergeCell ref="EZ44:EZ47"/>
+    <mergeCell ref="FA44:FA47"/>
+    <mergeCell ref="FB44:FB47"/>
+    <mergeCell ref="FC44:FC47"/>
+    <mergeCell ref="FD44:FD47"/>
+    <mergeCell ref="FE44:FE47"/>
+    <mergeCell ref="FF44:FF47"/>
+    <mergeCell ref="FG44:FG47"/>
+    <mergeCell ref="FH44:FH47"/>
+    <mergeCell ref="EQ44:EQ47"/>
+    <mergeCell ref="ER44:ER47"/>
+    <mergeCell ref="ES44:ES47"/>
+    <mergeCell ref="ET44:ET47"/>
+    <mergeCell ref="EU44:EU47"/>
+    <mergeCell ref="EV44:EV47"/>
+    <mergeCell ref="EW44:EW47"/>
+    <mergeCell ref="EX44:EX47"/>
+    <mergeCell ref="EY44:EY47"/>
+    <mergeCell ref="EH44:EH47"/>
+    <mergeCell ref="EI44:EI47"/>
+    <mergeCell ref="EJ44:EJ47"/>
+    <mergeCell ref="EK44:EK47"/>
+    <mergeCell ref="EL44:EL47"/>
+    <mergeCell ref="EM44:EM47"/>
+    <mergeCell ref="EN44:EN47"/>
+    <mergeCell ref="EO44:EO47"/>
+    <mergeCell ref="EP44:EP47"/>
+    <mergeCell ref="DY44:DY47"/>
+    <mergeCell ref="DZ44:DZ47"/>
+    <mergeCell ref="EA44:EA47"/>
+    <mergeCell ref="EB44:EB47"/>
+    <mergeCell ref="EC44:EC47"/>
+    <mergeCell ref="ED44:ED47"/>
+    <mergeCell ref="EE44:EE47"/>
+    <mergeCell ref="EF44:EF47"/>
+    <mergeCell ref="EG44:EG47"/>
+    <mergeCell ref="DP44:DP47"/>
+    <mergeCell ref="DQ44:DQ47"/>
+    <mergeCell ref="DR44:DR47"/>
+    <mergeCell ref="DS44:DS47"/>
+    <mergeCell ref="DT44:DT47"/>
+    <mergeCell ref="DU44:DU47"/>
+    <mergeCell ref="DV44:DV47"/>
+    <mergeCell ref="DW44:DW47"/>
+    <mergeCell ref="DX44:DX47"/>
+    <mergeCell ref="DG44:DG47"/>
+    <mergeCell ref="DH44:DH47"/>
+    <mergeCell ref="DI44:DI47"/>
+    <mergeCell ref="DJ44:DJ47"/>
+    <mergeCell ref="DK44:DK47"/>
+    <mergeCell ref="DL44:DL47"/>
+    <mergeCell ref="DM44:DM47"/>
+    <mergeCell ref="DN44:DN47"/>
+    <mergeCell ref="DO44:DO47"/>
+    <mergeCell ref="CX44:CX47"/>
+    <mergeCell ref="CY44:CY47"/>
+    <mergeCell ref="CZ44:CZ47"/>
+    <mergeCell ref="DA44:DA47"/>
+    <mergeCell ref="DB44:DB47"/>
+    <mergeCell ref="DC44:DC47"/>
+    <mergeCell ref="DD44:DD47"/>
+    <mergeCell ref="DE44:DE47"/>
+    <mergeCell ref="DF44:DF47"/>
+    <mergeCell ref="CO44:CO47"/>
+    <mergeCell ref="CP44:CP47"/>
+    <mergeCell ref="CQ44:CQ47"/>
+    <mergeCell ref="CR44:CR47"/>
+    <mergeCell ref="CS44:CS47"/>
+    <mergeCell ref="CT44:CT47"/>
+    <mergeCell ref="CU44:CU47"/>
+    <mergeCell ref="CV44:CV47"/>
+    <mergeCell ref="CW44:CW47"/>
+    <mergeCell ref="CF44:CF47"/>
+    <mergeCell ref="CG44:CG47"/>
+    <mergeCell ref="CH44:CH47"/>
+    <mergeCell ref="CI44:CI47"/>
+    <mergeCell ref="CJ44:CJ47"/>
+    <mergeCell ref="CK44:CK47"/>
+    <mergeCell ref="CL44:CL47"/>
+    <mergeCell ref="CM44:CM47"/>
+    <mergeCell ref="CN44:CN47"/>
+    <mergeCell ref="BW44:BW47"/>
+    <mergeCell ref="BX44:BX47"/>
+    <mergeCell ref="BY44:BY47"/>
+    <mergeCell ref="BZ44:BZ47"/>
+    <mergeCell ref="CA44:CA47"/>
+    <mergeCell ref="CB44:CB47"/>
+    <mergeCell ref="CC44:CC47"/>
+    <mergeCell ref="CD44:CD47"/>
+    <mergeCell ref="CE44:CE47"/>
+    <mergeCell ref="BN44:BN47"/>
+    <mergeCell ref="BO44:BO47"/>
+    <mergeCell ref="BP44:BP47"/>
+    <mergeCell ref="BQ44:BQ47"/>
+    <mergeCell ref="BR44:BR47"/>
+    <mergeCell ref="BS44:BS47"/>
+    <mergeCell ref="BT44:BT47"/>
+    <mergeCell ref="BU44:BU47"/>
+    <mergeCell ref="BV44:BV47"/>
+    <mergeCell ref="BE44:BE47"/>
+    <mergeCell ref="BF44:BF47"/>
+    <mergeCell ref="BG44:BG47"/>
+    <mergeCell ref="BH44:BH47"/>
+    <mergeCell ref="BI44:BI47"/>
+    <mergeCell ref="BJ44:BJ47"/>
+    <mergeCell ref="BK44:BK47"/>
+    <mergeCell ref="BL44:BL47"/>
+    <mergeCell ref="BM44:BM47"/>
+    <mergeCell ref="AV44:AV47"/>
+    <mergeCell ref="AW44:AW47"/>
+    <mergeCell ref="AX44:AX47"/>
+    <mergeCell ref="AY44:AY47"/>
+    <mergeCell ref="AZ44:AZ47"/>
+    <mergeCell ref="BA44:BA47"/>
+    <mergeCell ref="BB44:BB47"/>
+    <mergeCell ref="BC44:BC47"/>
+    <mergeCell ref="BD44:BD47"/>
+    <mergeCell ref="AM44:AM47"/>
+    <mergeCell ref="AN44:AN47"/>
+    <mergeCell ref="AO44:AO47"/>
+    <mergeCell ref="AP44:AP47"/>
+    <mergeCell ref="AQ44:AQ47"/>
+    <mergeCell ref="AR44:AR47"/>
+    <mergeCell ref="AS44:AS47"/>
+    <mergeCell ref="AT44:AT47"/>
+    <mergeCell ref="AU44:AU47"/>
+    <mergeCell ref="AD44:AD47"/>
+    <mergeCell ref="AE44:AE47"/>
+    <mergeCell ref="AF44:AF47"/>
+    <mergeCell ref="AG44:AG47"/>
+    <mergeCell ref="AH44:AH47"/>
+    <mergeCell ref="AI44:AI47"/>
+    <mergeCell ref="AJ44:AJ47"/>
+    <mergeCell ref="AK44:AK47"/>
+    <mergeCell ref="AL44:AL47"/>
+    <mergeCell ref="U44:U47"/>
+    <mergeCell ref="V44:V47"/>
+    <mergeCell ref="W44:W47"/>
+    <mergeCell ref="X44:X47"/>
+    <mergeCell ref="Y44:Y47"/>
+    <mergeCell ref="Z44:Z47"/>
+    <mergeCell ref="AA44:AA47"/>
+    <mergeCell ref="AB44:AB47"/>
+    <mergeCell ref="AC44:AC47"/>
+    <mergeCell ref="L44:L47"/>
+    <mergeCell ref="M44:M47"/>
+    <mergeCell ref="N44:N47"/>
+    <mergeCell ref="O44:O47"/>
+    <mergeCell ref="P44:P47"/>
+    <mergeCell ref="Q44:Q47"/>
+    <mergeCell ref="R44:R47"/>
+    <mergeCell ref="S44:S47"/>
+    <mergeCell ref="T44:T47"/>
+    <mergeCell ref="D44:D47"/>
+    <mergeCell ref="E44:E47"/>
+    <mergeCell ref="F44:F47"/>
+    <mergeCell ref="G44:G47"/>
+    <mergeCell ref="H44:H47"/>
+    <mergeCell ref="I44:I47"/>
+    <mergeCell ref="J44:J47"/>
+    <mergeCell ref="K44:K47"/>
+    <mergeCell ref="H36:H39"/>
+    <mergeCell ref="I36:I39"/>
+    <mergeCell ref="J36:J39"/>
+    <mergeCell ref="K36:K39"/>
+    <mergeCell ref="L36:L39"/>
+    <mergeCell ref="M36:M39"/>
+    <mergeCell ref="C36:C39"/>
+    <mergeCell ref="D36:D39"/>
+    <mergeCell ref="E36:E39"/>
+    <mergeCell ref="F36:F39"/>
+    <mergeCell ref="G36:G39"/>
+    <mergeCell ref="T36:T39"/>
+    <mergeCell ref="U36:U39"/>
+    <mergeCell ref="V36:V39"/>
+    <mergeCell ref="W36:W39"/>
+    <mergeCell ref="X36:X39"/>
+    <mergeCell ref="Y36:Y39"/>
+    <mergeCell ref="N36:N39"/>
+    <mergeCell ref="O36:O39"/>
+    <mergeCell ref="P36:P39"/>
+    <mergeCell ref="Q36:Q39"/>
+    <mergeCell ref="R36:R39"/>
+    <mergeCell ref="S36:S39"/>
+    <mergeCell ref="AF36:AF39"/>
+    <mergeCell ref="AG36:AG39"/>
+    <mergeCell ref="AH36:AH39"/>
+    <mergeCell ref="AI36:AI39"/>
+    <mergeCell ref="AJ36:AJ39"/>
+    <mergeCell ref="AK36:AK39"/>
+    <mergeCell ref="Z36:Z39"/>
+    <mergeCell ref="AA36:AA39"/>
+    <mergeCell ref="AB36:AB39"/>
+    <mergeCell ref="AC36:AC39"/>
+    <mergeCell ref="AD36:AD39"/>
+    <mergeCell ref="AE36:AE39"/>
+    <mergeCell ref="AR36:AR39"/>
+    <mergeCell ref="AS36:AS39"/>
+    <mergeCell ref="AT36:AT39"/>
+    <mergeCell ref="AU36:AU39"/>
+    <mergeCell ref="AV36:AV39"/>
+    <mergeCell ref="AW36:AW39"/>
+    <mergeCell ref="AL36:AL39"/>
+    <mergeCell ref="AM36:AM39"/>
+    <mergeCell ref="AN36:AN39"/>
+    <mergeCell ref="AO36:AO39"/>
+    <mergeCell ref="AP36:AP39"/>
+    <mergeCell ref="AQ36:AQ39"/>
+    <mergeCell ref="BD36:BD39"/>
+    <mergeCell ref="BE36:BE39"/>
+    <mergeCell ref="BF36:BF39"/>
+    <mergeCell ref="BG36:BG39"/>
+    <mergeCell ref="BH36:BH39"/>
+    <mergeCell ref="BI36:BI39"/>
+    <mergeCell ref="AX36:AX39"/>
+    <mergeCell ref="AY36:AY39"/>
+    <mergeCell ref="AZ36:AZ39"/>
+    <mergeCell ref="BA36:BA39"/>
+    <mergeCell ref="BB36:BB39"/>
+    <mergeCell ref="BC36:BC39"/>
+    <mergeCell ref="BP36:BP39"/>
+    <mergeCell ref="BQ36:BQ39"/>
+    <mergeCell ref="BR36:BR39"/>
+    <mergeCell ref="BS36:BS39"/>
+    <mergeCell ref="BT36:BT39"/>
+    <mergeCell ref="BU36:BU39"/>
+    <mergeCell ref="BJ36:BJ39"/>
+    <mergeCell ref="BK36:BK39"/>
+    <mergeCell ref="BL36:BL39"/>
+    <mergeCell ref="BM36:BM39"/>
+    <mergeCell ref="BN36:BN39"/>
+    <mergeCell ref="BO36:BO39"/>
+    <mergeCell ref="CB36:CB39"/>
+    <mergeCell ref="CC36:CC39"/>
+    <mergeCell ref="CD36:CD39"/>
+    <mergeCell ref="CE36:CE39"/>
+    <mergeCell ref="CF36:CF39"/>
+    <mergeCell ref="CG36:CG39"/>
+    <mergeCell ref="BV36:BV39"/>
+    <mergeCell ref="BW36:BW39"/>
+    <mergeCell ref="BX36:BX39"/>
+    <mergeCell ref="BY36:BY39"/>
+    <mergeCell ref="BZ36:BZ39"/>
+    <mergeCell ref="CA36:CA39"/>
+    <mergeCell ref="CN36:CN39"/>
+    <mergeCell ref="CO36:CO39"/>
+    <mergeCell ref="CP36:CP39"/>
+    <mergeCell ref="CQ36:CQ39"/>
+    <mergeCell ref="CR36:CR39"/>
+    <mergeCell ref="CS36:CS39"/>
+    <mergeCell ref="CH36:CH39"/>
+    <mergeCell ref="CI36:CI39"/>
+    <mergeCell ref="CJ36:CJ39"/>
+    <mergeCell ref="CK36:CK39"/>
+    <mergeCell ref="CL36:CL39"/>
+    <mergeCell ref="CM36:CM39"/>
+    <mergeCell ref="CZ36:CZ39"/>
+    <mergeCell ref="DA36:DA39"/>
+    <mergeCell ref="DB36:DB39"/>
+    <mergeCell ref="DC36:DC39"/>
+    <mergeCell ref="DD36:DD39"/>
+    <mergeCell ref="DE36:DE39"/>
+    <mergeCell ref="CT36:CT39"/>
+    <mergeCell ref="CU36:CU39"/>
+    <mergeCell ref="CV36:CV39"/>
+    <mergeCell ref="CW36:CW39"/>
+    <mergeCell ref="CX36:CX39"/>
+    <mergeCell ref="CY36:CY39"/>
+    <mergeCell ref="DL36:DL39"/>
+    <mergeCell ref="DM36:DM39"/>
+    <mergeCell ref="DN36:DN39"/>
+    <mergeCell ref="DO36:DO39"/>
+    <mergeCell ref="DP36:DP39"/>
+    <mergeCell ref="DQ36:DQ39"/>
+    <mergeCell ref="DF36:DF39"/>
+    <mergeCell ref="DG36:DG39"/>
+    <mergeCell ref="DH36:DH39"/>
+    <mergeCell ref="DI36:DI39"/>
+    <mergeCell ref="DJ36:DJ39"/>
+    <mergeCell ref="DK36:DK39"/>
+    <mergeCell ref="DX36:DX39"/>
+    <mergeCell ref="DY36:DY39"/>
+    <mergeCell ref="DZ36:DZ39"/>
+    <mergeCell ref="EA36:EA39"/>
+    <mergeCell ref="EB36:EB39"/>
+    <mergeCell ref="EC36:EC39"/>
+    <mergeCell ref="DR36:DR39"/>
+    <mergeCell ref="DS36:DS39"/>
+    <mergeCell ref="DT36:DT39"/>
+    <mergeCell ref="DU36:DU39"/>
+    <mergeCell ref="DV36:DV39"/>
+    <mergeCell ref="DW36:DW39"/>
+    <mergeCell ref="EJ36:EJ39"/>
+    <mergeCell ref="EK36:EK39"/>
+    <mergeCell ref="EL36:EL39"/>
+    <mergeCell ref="EM36:EM39"/>
+    <mergeCell ref="EN36:EN39"/>
+    <mergeCell ref="EO36:EO39"/>
+    <mergeCell ref="ED36:ED39"/>
+    <mergeCell ref="EE36:EE39"/>
+    <mergeCell ref="EF36:EF39"/>
+    <mergeCell ref="EG36:EG39"/>
+    <mergeCell ref="EH36:EH39"/>
+    <mergeCell ref="EI36:EI39"/>
+    <mergeCell ref="EV36:EV39"/>
+    <mergeCell ref="EW36:EW39"/>
+    <mergeCell ref="EX36:EX39"/>
+    <mergeCell ref="EY36:EY39"/>
+    <mergeCell ref="EZ36:EZ39"/>
+    <mergeCell ref="FA36:FA39"/>
+    <mergeCell ref="EP36:EP39"/>
+    <mergeCell ref="EQ36:EQ39"/>
+    <mergeCell ref="ER36:ER39"/>
+    <mergeCell ref="ES36:ES39"/>
+    <mergeCell ref="ET36:ET39"/>
+    <mergeCell ref="EU36:EU39"/>
+    <mergeCell ref="FH36:FH39"/>
+    <mergeCell ref="FI36:FI39"/>
+    <mergeCell ref="FJ36:FJ39"/>
+    <mergeCell ref="FK36:FK39"/>
+    <mergeCell ref="FL36:FL39"/>
+    <mergeCell ref="FM36:FM39"/>
+    <mergeCell ref="FB36:FB39"/>
+    <mergeCell ref="FC36:FC39"/>
+    <mergeCell ref="FD36:FD39"/>
+    <mergeCell ref="FE36:FE39"/>
+    <mergeCell ref="FF36:FF39"/>
+    <mergeCell ref="FG36:FG39"/>
+    <mergeCell ref="FT36:FT39"/>
+    <mergeCell ref="FU36:FU39"/>
+    <mergeCell ref="FV36:FV39"/>
+    <mergeCell ref="FW36:FW39"/>
+    <mergeCell ref="FX36:FX39"/>
+    <mergeCell ref="FY36:FY39"/>
+    <mergeCell ref="FN36:FN39"/>
+    <mergeCell ref="FO36:FO39"/>
+    <mergeCell ref="FP36:FP39"/>
+    <mergeCell ref="FQ36:FQ39"/>
+    <mergeCell ref="FR36:FR39"/>
+    <mergeCell ref="FS36:FS39"/>
+    <mergeCell ref="GF36:GF39"/>
+    <mergeCell ref="GG36:GG39"/>
+    <mergeCell ref="GH36:GH39"/>
+    <mergeCell ref="GI36:GI39"/>
+    <mergeCell ref="GJ36:GJ39"/>
+    <mergeCell ref="GK36:GK39"/>
+    <mergeCell ref="FZ36:FZ39"/>
+    <mergeCell ref="GA36:GA39"/>
+    <mergeCell ref="GB36:GB39"/>
+    <mergeCell ref="GC36:GC39"/>
+    <mergeCell ref="GD36:GD39"/>
+    <mergeCell ref="GE36:GE39"/>
+    <mergeCell ref="GR36:GR39"/>
+    <mergeCell ref="GS36:GS39"/>
+    <mergeCell ref="GT36:GT39"/>
+    <mergeCell ref="GU36:GU39"/>
+    <mergeCell ref="GV36:GV39"/>
+    <mergeCell ref="GW36:GW39"/>
+    <mergeCell ref="GL36:GL39"/>
+    <mergeCell ref="GM36:GM39"/>
+    <mergeCell ref="GN36:GN39"/>
+    <mergeCell ref="GO36:GO39"/>
+    <mergeCell ref="GP36:GP39"/>
+    <mergeCell ref="GQ36:GQ39"/>
+    <mergeCell ref="HD36:HD39"/>
+    <mergeCell ref="HE36:HE39"/>
+    <mergeCell ref="HF36:HF39"/>
+    <mergeCell ref="HG36:HG39"/>
+    <mergeCell ref="HH36:HH39"/>
+    <mergeCell ref="HI36:HI39"/>
+    <mergeCell ref="GX36:GX39"/>
+    <mergeCell ref="GY36:GY39"/>
+    <mergeCell ref="GZ36:GZ39"/>
+    <mergeCell ref="HA36:HA39"/>
+    <mergeCell ref="HB36:HB39"/>
+    <mergeCell ref="HC36:HC39"/>
+    <mergeCell ref="HP36:HP39"/>
+    <mergeCell ref="HQ36:HQ39"/>
+    <mergeCell ref="HR36:HR39"/>
+    <mergeCell ref="HS36:HS39"/>
+    <mergeCell ref="HT36:HT39"/>
+    <mergeCell ref="HU36:HU39"/>
+    <mergeCell ref="HJ36:HJ39"/>
+    <mergeCell ref="HK36:HK39"/>
+    <mergeCell ref="HL36:HL39"/>
+    <mergeCell ref="HM36:HM39"/>
+    <mergeCell ref="HN36:HN39"/>
+    <mergeCell ref="HO36:HO39"/>
+    <mergeCell ref="IB36:IB39"/>
+    <mergeCell ref="IC36:IC39"/>
+    <mergeCell ref="ID36:ID39"/>
+    <mergeCell ref="IE36:IE39"/>
+    <mergeCell ref="IF36:IF39"/>
+    <mergeCell ref="IG36:IG39"/>
+    <mergeCell ref="HV36:HV39"/>
+    <mergeCell ref="HW36:HW39"/>
+    <mergeCell ref="HX36:HX39"/>
+    <mergeCell ref="HY36:HY39"/>
+    <mergeCell ref="HZ36:HZ39"/>
+    <mergeCell ref="IA36:IA39"/>
+    <mergeCell ref="IN36:IN39"/>
+    <mergeCell ref="IO36:IO39"/>
+    <mergeCell ref="IP36:IP39"/>
+    <mergeCell ref="IQ36:IQ39"/>
+    <mergeCell ref="IR36:IR39"/>
+    <mergeCell ref="IH36:IH39"/>
+    <mergeCell ref="II36:II39"/>
+    <mergeCell ref="IJ36:IJ39"/>
+    <mergeCell ref="IK36:IK39"/>
+    <mergeCell ref="IL36:IL39"/>
+    <mergeCell ref="IM36:IM39"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11267,29 +11267,29 @@
   <sheetData>
     <row r="1" spans="1:12" ht="42" x14ac:dyDescent="0.15">
       <c r="A1" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>109</v>
       </c>
       <c r="H1" s="6"/>
       <c r="I1" s="45" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J1" s="6"/>
       <c r="K1" s="6"/>
@@ -11297,29 +11297,29 @@
     </row>
     <row r="2" spans="1:12" ht="14" x14ac:dyDescent="0.15">
       <c r="A2" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B2" s="9">
         <v>1</v>
       </c>
       <c r="C2" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="E2" s="10" t="s">
         <v>112</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>113</v>
       </c>
       <c r="F2" s="9">
         <v>1</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H2" s="6"/>
       <c r="I2" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
@@ -11327,27 +11327,27 @@
     </row>
     <row r="3" spans="1:12" ht="14" x14ac:dyDescent="0.15">
       <c r="A3" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B3" s="9">
         <v>2</v>
       </c>
       <c r="C3" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>115</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>116</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="9">
         <v>2</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
@@ -11355,27 +11355,27 @@
     </row>
     <row r="4" spans="1:12" ht="14" x14ac:dyDescent="0.15">
       <c r="A4" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B4" s="9">
         <v>3</v>
       </c>
       <c r="C4" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>119</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>120</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="9">
         <v>3</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H4" s="6"/>
       <c r="I4" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
@@ -11383,27 +11383,27 @@
     </row>
     <row r="5" spans="1:12" ht="14" x14ac:dyDescent="0.15">
       <c r="A5" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B5" s="9">
         <v>4</v>
       </c>
       <c r="C5" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>123</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>124</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="9">
         <v>4</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H5" s="6"/>
       <c r="I5" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
@@ -11411,23 +11411,23 @@
     </row>
     <row r="6" spans="1:12" ht="14" x14ac:dyDescent="0.15">
       <c r="A6" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B6" s="9">
         <v>5</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="9">
         <v>5</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
@@ -11437,23 +11437,23 @@
     </row>
     <row r="7" spans="1:12" ht="14" x14ac:dyDescent="0.15">
       <c r="A7" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B7" s="9">
         <v>6</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>130</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>131</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="9">
         <v>6</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
@@ -11463,23 +11463,23 @@
     </row>
     <row r="8" spans="1:12" ht="14" x14ac:dyDescent="0.15">
       <c r="A8" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B8" s="9">
         <v>7</v>
       </c>
       <c r="C8" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>134</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>135</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="9">
         <v>7</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
@@ -11489,27 +11489,27 @@
     </row>
     <row r="9" spans="1:12" ht="14" x14ac:dyDescent="0.15">
       <c r="A9" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B9" s="9">
         <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="9">
         <v>8</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H9" s="6"/>
       <c r="I9" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
@@ -11517,11 +11517,11 @@
     </row>
     <row r="10" spans="1:12" ht="28" x14ac:dyDescent="0.15">
       <c r="A10" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
@@ -11532,16 +11532,16 @@
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
       <c r="L10" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="28" x14ac:dyDescent="0.15">
       <c r="A11" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
@@ -11552,14 +11552,14 @@
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
       <c r="L11" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D12" s="7"/>
       <c r="E12" s="7"/>
@@ -11575,7 +11575,7 @@
       <c r="A13" s="6"/>
       <c r="B13" s="11"/>
       <c r="C13" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
@@ -11591,7 +11591,7 @@
       <c r="A14" s="12"/>
       <c r="B14" s="6"/>
       <c r="C14" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D14" s="7"/>
       <c r="E14" s="7"/>
@@ -11607,7 +11607,7 @@
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
@@ -11621,7 +11621,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A16" s="49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B16" s="46"/>
       <c r="C16" s="46"/>
@@ -11637,10 +11637,10 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A17" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C17" s="6"/>
       <c r="D17" s="48"/>
@@ -11655,10 +11655,10 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A18" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="48"/>
@@ -11673,10 +11673,10 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A19" s="12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="48"/>
@@ -11691,10 +11691,10 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A20" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="48"/>
@@ -11709,10 +11709,10 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A21" s="12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="48"/>
@@ -11727,10 +11727,10 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A22" s="12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="48"/>
@@ -11745,10 +11745,10 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A23" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B23" s="8" t="s">
         <v>152</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>153</v>
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="7"/>
@@ -11763,7 +11763,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A24" s="49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B24" s="46"/>
       <c r="C24" s="46"/>
@@ -11779,7 +11779,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A25" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -11795,7 +11795,7 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A26" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="7"/>
@@ -11810,7 +11810,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A27" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="7"/>
@@ -11825,7 +11825,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A28" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="7"/>
@@ -11840,7 +11840,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A29" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="7"/>
@@ -11855,7 +11855,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A30" s="49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B30" s="46"/>
       <c r="C30" s="46"/>
@@ -11871,10 +11871,10 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A31" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C31" s="6"/>
       <c r="D31" s="7"/>
@@ -11889,10 +11889,10 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A32" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="7"/>
@@ -11907,10 +11907,10 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A33" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C33" s="6"/>
       <c r="D33" s="7"/>
@@ -11925,10 +11925,10 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A34" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="7"/>
@@ -11943,10 +11943,10 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A35" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C35" s="6"/>
       <c r="D35" s="7"/>
@@ -11961,10 +11961,10 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A36" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="7"/>
@@ -11979,10 +11979,10 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A37" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C37" s="6"/>
       <c r="D37" s="7"/>
@@ -11997,10 +11997,10 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A38" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="7"/>
@@ -12015,10 +12015,10 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A39" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C39" s="6"/>
       <c r="D39" s="7"/>
@@ -12033,10 +12033,10 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A40" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="7"/>
@@ -12051,10 +12051,10 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A41" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C41" s="6"/>
       <c r="D41" s="7"/>
@@ -12069,10 +12069,10 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A42" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="7"/>

</xml_diff>